<commit_message>
added script to start scheduler
</commit_message>
<xml_diff>
--- a/hardware/manufacture/v1.0.1/bom.xlsx
+++ b/hardware/manufacture/v1.0.1/bom.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isuruceanu/workspace/projects/valvos.dev/aqua-eq8/hardware/manufacture/v1.0.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB7C375-5ECA-FF4A-8544-71DB7DB3B6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BC8879-B9BD-7945-9ADD-465C41DD1335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-360" windowWidth="38400" windowHeight="19320" xr2:uid="{B54978BE-B69C-324E-BE22-B13E158F1B1C}"/>
+    <workbookView xWindow="38860" yWindow="2240" windowWidth="28040" windowHeight="17180" xr2:uid="{2747D124-8B25-E849-B842-CB5CB20BDDCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="hw_controller" localSheetId="0">Sheet1!$A$1:$H$47</definedName>
+    <definedName name="hw_controller" localSheetId="0">Sheet1!$A$1:$G$38</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,7 +43,7 @@
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
-  <connection id="1" xr16:uid="{A95BEAB7-E63C-6242-89AD-4A077C595B7E}" name="hw-controller" type="6" refreshedVersion="8" background="1" saveData="1">
+  <connection id="1" xr16:uid="{E731B504-2D54-9643-86B3-B5ECFF383A87}" name="hw-controller" type="6" refreshedVersion="8" background="1" saveData="1">
     <textPr codePage="10000" sourceFile="/Users/isuruceanu/workspace/projects/valvos.dev/aqua-eq8/hardware/manufacture/v1.0.1/hw-controller.csv" semicolon="1">
       <textFields count="8">
         <textField/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="95">
   <si>
     <t>Id</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Designation</t>
   </si>
   <si>
-    <t>Supplier and ref</t>
-  </si>
-  <si>
     <t>BR1</t>
   </si>
   <si>
@@ -147,6 +144,9 @@
     <t>C17</t>
   </si>
   <si>
+    <t>12pF</t>
+  </si>
+  <si>
     <t>C19</t>
   </si>
   <si>
@@ -198,6 +198,9 @@
     <t>J1</t>
   </si>
   <si>
+    <t>PinHeader_2x03_P1.27mm_Vertical_SMD</t>
+  </si>
+  <si>
     <t>Conn_02x03_Odd_Even</t>
   </si>
   <si>
@@ -282,72 +285,9 @@
     <t>50k</t>
   </si>
   <si>
-    <t>S1</t>
-  </si>
-  <si>
     <t>228EMVARGBFR</t>
   </si>
   <si>
-    <t>RGBFR_CH1</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>RGBFR_CH2</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t>RGBFR_CH3</t>
-  </si>
-  <si>
-    <t>S4</t>
-  </si>
-  <si>
-    <t>RGBFR_CH4</t>
-  </si>
-  <si>
-    <t>S5</t>
-  </si>
-  <si>
-    <t>RGBFR_CH5</t>
-  </si>
-  <si>
-    <t>S6</t>
-  </si>
-  <si>
-    <t>RGBFR_CH6</t>
-  </si>
-  <si>
-    <t>S7</t>
-  </si>
-  <si>
-    <t>RGBFR_CH7</t>
-  </si>
-  <si>
-    <t>S8</t>
-  </si>
-  <si>
-    <t>RGBFR_CH8</t>
-  </si>
-  <si>
-    <t>S9</t>
-  </si>
-  <si>
-    <t>RGBFR_STATUS</t>
-  </si>
-  <si>
-    <t>TP1, TP2, TP3, TP4</t>
-  </si>
-  <si>
-    <t>TP_1_27</t>
-  </si>
-  <si>
-    <t>~</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -402,10 +342,10 @@
     <t>ACS725xLCTR-20AB</t>
   </si>
   <si>
-    <t>12pF</t>
-  </si>
-  <si>
-    <t>PinHeader_2x03_P1.27mm_Vertical_SMD</t>
+    <t>S1-S9</t>
+  </si>
+  <si>
+    <t>RGBFR_CH1_8_Status</t>
   </si>
 </sst>
 </file>
@@ -441,11 +381,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,7 +405,7 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="hw-controller" connectionId="1" xr16:uid="{7D7C7838-93A8-0D41-870E-AAE9A024CD7B}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="hw-controller" connectionId="1" xr16:uid="{284A7AA8-429F-284E-B7DC-7D83B367E1CF}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -783,19 +724,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9E910B1-A80A-674A-B821-22C1B20D8CB5}">
-  <dimension ref="A1:F47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{657256F7-FC0F-1949-97DC-409007174278}">
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5" customWidth="1"/>
+    <col min="3" max="3" width="57.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.1640625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -808,167 +748,164 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
         <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
         <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
       </c>
       <c r="D4">
         <v>8</v>
       </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
         <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
       </c>
       <c r="D5">
         <v>2</v>
       </c>
-      <c r="E5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E7" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8">
         <v>4</v>
       </c>
-      <c r="E8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E8" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -976,16 +913,16 @@
         <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
-      <c r="E11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -993,16 +930,16 @@
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
-      <c r="E12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1010,16 +947,16 @@
         <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1032,11 +969,11 @@
       <c r="D14">
         <v>1</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1049,11 +986,11 @@
       <c r="D15">
         <v>8</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1066,7 +1003,7 @@
       <c r="D16">
         <v>1</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1083,7 +1020,7 @@
       <c r="D17">
         <v>1</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1095,30 +1032,30 @@
         <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>114</v>
+        <v>45</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="E18" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="E18" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" s="1" t="s">
         <v>47</v>
       </c>
+      <c r="C19" t="s">
+        <v>48</v>
+      </c>
       <c r="D19">
         <v>1</v>
       </c>
-      <c r="E19" t="s">
-        <v>48</v>
+      <c r="E19" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1126,16 +1063,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
-      <c r="E20" t="s">
-        <v>51</v>
+      <c r="E20" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1143,16 +1080,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="E21" t="s">
-        <v>54</v>
+      <c r="E21" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1160,32 +1097,32 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D22">
         <v>6</v>
       </c>
-      <c r="E22" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="E22" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D23">
         <v>24</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="2">
         <v>470</v>
       </c>
     </row>
@@ -1194,15 +1131,15 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D24">
         <v>8</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="2">
         <v>330</v>
       </c>
     </row>
@@ -1211,15 +1148,15 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D25">
         <v>1</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="2">
         <v>33</v>
       </c>
     </row>
@@ -1228,15 +1165,15 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D26">
         <v>8</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="2">
         <v>160</v>
       </c>
     </row>
@@ -1245,16 +1182,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D27">
         <v>7</v>
       </c>
-      <c r="E27" t="s">
-        <v>64</v>
+      <c r="E27" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1262,15 +1199,15 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C28" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D28">
         <v>3</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="2">
         <v>150</v>
       </c>
     </row>
@@ -1279,16 +1216,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C29" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
-      <c r="E29" t="s">
-        <v>67</v>
+      <c r="E29" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -1296,16 +1233,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D30">
         <v>1</v>
       </c>
-      <c r="E30" t="s">
-        <v>70</v>
+      <c r="E30" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1313,16 +1250,16 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C31" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D31">
         <v>1</v>
       </c>
-      <c r="E31" t="s">
-        <v>72</v>
+      <c r="E31" s="2" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1330,271 +1267,118 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="C32" t="s">
         <v>74</v>
       </c>
       <c r="D32">
-        <v>1</v>
-      </c>
-      <c r="E32" t="s">
-        <v>75</v>
+        <v>9</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" t="s">
         <v>76</v>
       </c>
-      <c r="C33" t="s">
-        <v>74</v>
-      </c>
       <c r="D33">
         <v>1</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="2" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B34" t="s">
         <v>78</v>
       </c>
       <c r="C34" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D34">
         <v>1</v>
       </c>
-      <c r="E34" t="s">
-        <v>79</v>
+      <c r="E34" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D35">
-        <v>1</v>
-      </c>
-      <c r="E35" t="s">
-        <v>81</v>
+        <v>2</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C36" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="D36">
-        <v>1</v>
-      </c>
-      <c r="E36" t="s">
-        <v>83</v>
+        <v>8</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="B37" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="D37">
         <v>1</v>
       </c>
-      <c r="E37" t="s">
-        <v>85</v>
+      <c r="E37" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="D38">
         <v>1</v>
       </c>
-      <c r="E38" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39" t="s">
-        <v>88</v>
-      </c>
-      <c r="C39" t="s">
-        <v>74</v>
-      </c>
-      <c r="D39">
-        <v>1</v>
-      </c>
-      <c r="E39" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40" t="s">
-        <v>90</v>
-      </c>
-      <c r="C40" t="s">
-        <v>74</v>
-      </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
-      <c r="E40" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="s">
+      <c r="E38" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="C41" t="s">
-        <v>93</v>
-      </c>
-      <c r="D41">
-        <v>4</v>
-      </c>
-      <c r="E41" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" t="s">
-        <v>95</v>
-      </c>
-      <c r="C42" t="s">
-        <v>96</v>
-      </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="E42" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43" t="s">
-        <v>98</v>
-      </c>
-      <c r="C43" t="s">
-        <v>99</v>
-      </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
-      <c r="E43" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44" t="s">
-        <v>101</v>
-      </c>
-      <c r="C44" t="s">
-        <v>102</v>
-      </c>
-      <c r="D44">
-        <v>2</v>
-      </c>
-      <c r="E44" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C45" t="s">
-        <v>105</v>
-      </c>
-      <c r="D45">
-        <v>8</v>
-      </c>
-      <c r="E45" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46" t="s">
-        <v>107</v>
-      </c>
-      <c r="C46" t="s">
-        <v>108</v>
-      </c>
-      <c r="D46">
-        <v>1</v>
-      </c>
-      <c r="E46" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47" t="s">
-        <v>110</v>
-      </c>
-      <c r="C47" t="s">
-        <v>111</v>
-      </c>
-      <c r="D47">
-        <v>1</v>
-      </c>
-      <c r="E47" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>